<commit_message>
revue des profils structure. ajout espace pour la lisibilité. changement de members en member. suppression du VS UAC non utilisé (#280) 6197c296fbe1a898e03d3bc616f444544e7709d8
</commit_message>
<xml_diff>
--- a/main/ig/CodeSystem-fr-core-cs-location-type.xlsx
+++ b/main/ig/CodeSystem-fr-core-cs-location-type.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-09T06:47:58+00:00</t>
+    <t>2026-02-11T16:15:37+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -183,7 +183,7 @@
     <t>LIT</t>
   </si>
   <si>
-    <t>lit</t>
+    <t>Lit</t>
   </si>
   <si>
     <t>PL_TECH</t>

</xml_diff>